<commit_message>
Remove items whose name starts with G
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016GtZZioynu6BNNHeRc885e
</commit_message>
<xml_diff>
--- a/shipments_by_item.xlsx
+++ b/shipments_by_item.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B122"/>
+  <dimension ref="A1:B89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -452,1440 +452,1044 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>4522646072136</t>
+          <t>4522646139150</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Ｇよだれ鶏（小）</t>
+          <t>Ｓよだれ鶏（小）</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>4522646139150</t>
+          <t>4522646089738</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ｓよだれ鶏（小）</t>
+          <t>味付海苔ツナマヨおにぎり５</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4522646089738</t>
+          <t>4522646102758</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>味付海苔ツナマヨおにぎり５</t>
+          <t>味付海苔エビマヨおにぎり３</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4522646102758</t>
+          <t>4522646105889</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>味付海苔エビマヨおにぎり３</t>
+          <t>赤飯おにぎりＰ</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4522646105889</t>
+          <t>4522646105902</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>赤飯おにぎりＰ</t>
+          <t>梅しそおにぎりＰ</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4522646105902</t>
+          <t>4522646106077</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>梅しそおにぎりＰ</t>
+          <t>梅ひじきおにぎりＰ</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>4522646106077</t>
+          <t>4522646106084</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>梅ひじきおにぎりＰ</t>
+          <t>鶏めしおにぎりＰ</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>4522646106084</t>
+          <t>4522646153484</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>鶏めしおにぎりＰ</t>
+          <t>わかめたっぷりおにぎりＰ２</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>4522646153484</t>
+          <t>4522646193305</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>わかめたっぷりおにぎりＰ２</t>
+          <t>あさり志ぐれおにぎり４</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>4522646193305</t>
+          <t>4522646193336</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>あさり志ぐれおにぎり４</t>
+          <t>明太子おにぎり４</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>4522646193336</t>
+          <t>4522646193619</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>明太子おにぎり４</t>
+          <t>鮭おにぎり６</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>4522646193619</t>
+          <t>4522646194111</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>鮭おにぎり６</t>
+          <t>しそ昆布おにぎり６</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>4522646194111</t>
+          <t>4522646194128</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>しそ昆布おにぎり６</t>
+          <t>梅おにぎり（種なし）５</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>4522646194128</t>
+          <t>4522646198904</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>梅おにぎり（種なし）５</t>
+          <t>おかかおにぎり５</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>4522646198904</t>
+          <t>4522646138931</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>おかかおにぎり５</t>
+          <t>Ｓ関西風やきそば２</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>2500543000000</t>
+          <t>2502910000000</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>まっしろミルクプリン</t>
+          <t>あじ南蛮漬け６</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>2506693000000</t>
+          <t>2559224000000</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>大人のコーヒーゼリー４</t>
+          <t>揚げだし豆腐４</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2534840000000</t>
+          <t>2563814000000</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>みかんの牛乳寒天（小）</t>
+          <t>ごった煮５</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2543462000000</t>
+          <t>2502011000000</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>まっしろミルクプリン小２</t>
+          <t>チキンカツカレー９</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>2543467000000</t>
+          <t>2516789000000</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>大人のコーヒーゼリー小２</t>
+          <t>かしわおにぎり２個入り５</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>2576849000000</t>
+          <t>2530008000000</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>みかんの牛乳寒天２</t>
+          <t>焼き飯４</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>4522646066593</t>
+          <t>2542780000000</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ｇまっしろミルクプリン</t>
+          <t>ミニ鶏そぼろ丼</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>4522646086850</t>
+          <t>2543367000000</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Ｇ大人のコーヒーゼリー４</t>
+          <t>おにぎりセット（鮭・昆）７</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>4522646130508</t>
+          <t>2548783000000</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ｓまっしろミルクプリン小２</t>
+          <t>塩おにぎり２個入り</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>4522646130645</t>
+          <t>2551499000000</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ｓ大人のコーヒーゼリー小２</t>
+          <t>鶏めしセット</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>4522646139167</t>
+          <t>2551557000000</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ｓみかんの牛乳寒天２</t>
+          <t>２６うなぎ飯</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>4522646139174</t>
+          <t>2553040000000</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Ｓまっしろミルクプリン</t>
+          <t>わかめごはんセット</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>4522646139181</t>
+          <t>2554872000000</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ｓ大人のコーヒーゼリー４</t>
+          <t>鶏めし幕の内弁当３</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>4522646138931</t>
+          <t>2556427000000</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ｓ関西風やきそば２</t>
+          <t>焼き飯＆チキン南蛮６</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>2502910000000</t>
+          <t>2556441000000</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>あじ南蛮漬け６</t>
+          <t>特選のり弁当１</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2559224000000</t>
+          <t>2556471000000</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>揚げだし豆腐４</t>
+          <t>洋食プレート（ピラフ）３</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2563814000000</t>
+          <t>2556976000000</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ごった煮５</t>
+          <t>塩おにぎり１０個２</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>4522646200447</t>
+          <t>2558048000000</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Ｇ揚げだし豆腐４</t>
+          <t>炒飯＆焼そば</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>2502011000000</t>
+          <t>2558056000000</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>チキンカツカレー９</t>
+          <t>しそひじきおにぎり２個</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2516789000000</t>
+          <t>2558809000000</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>かしわおにぎり２個入り５</t>
+          <t>自社製おはぎ２個４</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2530008000000</t>
+          <t>2558811000000</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>焼き飯４</t>
+          <t>自社製おはぎ３個６</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>2542780000000</t>
+          <t>2558814000000</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ミニ鶏そぼろ丼</t>
+          <t>きなこおはぎ２個４</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>2543367000000</t>
+          <t>2558828000000</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>おにぎりセット（鮭・昆）７</t>
+          <t>自社製おはぎアソート６</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2548783000000</t>
+          <t>2558875000000</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>塩おにぎり２個入り</t>
+          <t>小さなおはぎ（あんこ）５</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2551499000000</t>
+          <t>2558879000000</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>鶏めしセット</t>
+          <t>小さなおはぎ（きなこ）５</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2551557000000</t>
+          <t>2558887000000</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>２６うなぎ飯</t>
+          <t>自社製あん＆ホイップサンド</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2553040000000</t>
+          <t>2559215000000</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>わかめごはんセット</t>
+          <t>白いたっぷり玉子サンド</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2554872000000</t>
+          <t>2559614000000</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>鶏めし幕の内弁当３</t>
+          <t>たっぷり玉子＆ツナサンド２</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2556427000000</t>
+          <t>2559618000000</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>焼き飯＆チキン南蛮６</t>
+          <t>ハムレタスサンド</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>2556441000000</t>
+          <t>2561774000000</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>特選のり弁当１</t>
+          <t>肉肉ハンバーグ弁当</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>2556471000000</t>
+          <t>2562923000000</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>洋食プレート（ピラフ）３</t>
+          <t>塩おにぎりセット８</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>2556976000000</t>
+          <t>2562961000000</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>塩おにぎり１０個２</t>
+          <t>ちりめんおにぎりセット４</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>2558048000000</t>
+          <t>2563006000000</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>炒飯＆焼そば</t>
+          <t>梅しそおにぎりセット８</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>2558056000000</t>
+          <t>2563030000000</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>しそひじきおにぎり２個</t>
+          <t>銀鮭弁当５</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>2558809000000</t>
+          <t>2564314000000</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>自社製おはぎ２個４</t>
+          <t>２６栗おこわ２</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>2558811000000</t>
+          <t>2565596000000</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>自社製おはぎ３個６</t>
+          <t>ねぎ塩豚カルビ重（麦めし６</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>2558814000000</t>
+          <t>2570063000000</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>きなこおはぎ２個４</t>
+          <t>メンチカツサンド　１個</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>2558828000000</t>
+          <t>2571141000000</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>自社製おはぎアソート６</t>
+          <t>メンチカツ＆玉子サンド</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>2558875000000</t>
+          <t>2574221000000</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>小さなおはぎ（あんこ）５</t>
+          <t>牛焼肉重３</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>2558879000000</t>
+          <t>4522646130324</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>小さなおはぎ（きなこ）５</t>
+          <t>Ｓおにぎりセット（鮭・昆７</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>2558887000000</t>
+          <t>4522646138894</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>自社製あん＆ホイップサンド</t>
+          <t>Ｓ牛焼肉重３</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>2559215000000</t>
+          <t>4522646138900</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>白いたっぷり玉子サンド</t>
+          <t>Ｓねぎ塩豚カルビ（麦めし６</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>2559614000000</t>
+          <t>4522646190984</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>たっぷり玉子＆ツナサンド２</t>
+          <t>Ｓかしわおにぎり２個入り５</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>2559618000000</t>
+          <t>4522646190991</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ハムレタスサンド</t>
+          <t>Ｓ塩おにぎり２個入り</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>2561774000000</t>
+          <t>4522646191578</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>肉肉ハンバーグ弁当</t>
+          <t>Ｓ焼き飯４</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>2562923000000</t>
+          <t>4522646191592</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>塩おにぎりセット８</t>
+          <t>Ｓチキンカツカレー９</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>2562961000000</t>
+          <t>4522646191639</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ちりめんおにぎりセット４</t>
+          <t>Ｓ鶏めし幕の内弁当３</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>2563006000000</t>
+          <t>4522646198935</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>梅しそおにぎりセット８</t>
+          <t>Ｓ特選のり弁当１</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>2563030000000</t>
+          <t>4522646199444</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>銀鮭弁当５</t>
+          <t>Ｓ洋食プレート（ピラフ）３</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>2564314000000</t>
+          <t>4522646199451</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>２６栗おこわ２</t>
+          <t>Ｓ焼き飯＆チキン南蛮６</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>2565596000000</t>
+          <t>4522646199581</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ねぎ塩豚カルビ重（麦めし６</t>
+          <t>Ｓおはぎ２個４</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>2570063000000</t>
+          <t>4522646199598</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>メンチカツサンド　１個</t>
+          <t>Ｓおはぎ３個６</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>2571141000000</t>
+          <t>4522646199604</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>メンチカツ＆玉子サンド</t>
+          <t>Ｓきなこおはぎ２個４</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>2574221000000</t>
+          <t>4522646199611</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>牛焼肉重３</t>
+          <t>Ｓおはぎアソート６</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>4522646012941</t>
+          <t>4522646199635</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Ｇ塩おにぎり２個入り</t>
+          <t>Ｓ小さなおはぎ（あんこ）５</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>4522646016345</t>
+          <t>4522646199680</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Ｇねぎ塩豚カルビ（麦めし６</t>
+          <t>Ｓ小さなおはぎ（きなこ）５</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>4522646055979</t>
+          <t>4522646200461</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ｇ牛焼肉重３</t>
+          <t>Ｓ白いたっぷり玉子サンド</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>4522646071801</t>
+          <t>4522646201581</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Ｇチキンカツカレー９</t>
+          <t>Ｓ肉肉ハンバーグ弁当</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>4522646105216</t>
+          <t>4522646201888</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Ｇかしわおにぎり２個入り５</t>
+          <t>Ｓ銀鮭弁当５</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>4522646118292</t>
+          <t>2512464000000</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Ｇ焼き飯４</t>
+          <t>大盛ナポリタン</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>4522646129090</t>
+          <t>2532480000000</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Ｇミニ鶏そぼろ丼</t>
+          <t>関西風オムそば３</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>4522646130317</t>
+          <t>2532748000000</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ｇおにぎりセット（鮭・昆７</t>
+          <t>２６冷やし中華</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>4522646130324</t>
+          <t>2532787000000</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Ｓおにぎりセット（鮭・昆７</t>
+          <t>２６冷やし中華ミニ</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>4522646138894</t>
+          <t>2533587000000</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ｓ牛焼肉重３</t>
+          <t>２６冷やしきつねうどん</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>4522646138900</t>
+          <t>2551178000000</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Ｓねぎ塩豚カルビ（麦めし６</t>
+          <t>太麺ナポリタン２</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>4522646190984</t>
+          <t>2557960000000</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Ｓかしわおにぎり２個入り５</t>
+          <t>関西風焼きそば３</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>4522646190991</t>
+          <t>2571104000000</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Ｓ塩おにぎり２個入り</t>
+          <t>２６きつねうどん</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>4522646191578</t>
+          <t>2571107000000</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Ｓ焼き飯４</t>
+          <t>２６きつねうどん（小）</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>4522646191592</t>
+          <t>4522646138672</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Ｓチキンカツカレー９</t>
+          <t>Ｓ大盛ナポリタン</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>4522646191639</t>
+          <t>4522646138917</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Ｓ鶏めし幕の内弁当３</t>
+          <t>Ｓ関西風オムそば３</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>4522646198911</t>
+          <t>4522646150544</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Ｇ焼き飯＆チキン南蛮６</t>
+          <t>Ｓ太麺ナポリタン２</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>4522646198928</t>
+          <t>4522646199475</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Ｇ特選のり弁当１</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>4522646198935</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Ｓ特選のり弁当１</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>4522646199444</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>Ｓ洋食プレート（ピラフ）３</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>4522646199451</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>Ｓ焼き飯＆チキン南蛮６</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>4522646199581</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Ｓおはぎ２個４</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>4522646199598</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Ｓおはぎ３個６</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>4522646199604</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Ｓきなこおはぎ２個４</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>4522646199611</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Ｓおはぎアソート６</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>4522646199635</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Ｓ小さなおはぎ（あんこ）５</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>4522646199680</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Ｓ小さなおはぎ（きなこ）５</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>4522646199710</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Ｇおはぎ１個４</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>4522646200461</t>
-        </is>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Ｓ白いたっぷり玉子サンド</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>4522646200478</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Ｇ白いたっぷり玉子サンド</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>4522646201581</t>
-        </is>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Ｓ肉肉ハンバーグ弁当</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
-        <is>
-          <t>4522646201598</t>
-        </is>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Ｇ肉肉ハンバーグ弁当</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>4522646201789</t>
-        </is>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Ｇ塩おにぎりセット８</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>4522646201888</t>
-        </is>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Ｓ銀鮭弁当５</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>2512464000000</t>
-        </is>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>大盛ナポリタン</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>2532480000000</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>関西風オムそば３</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>2532748000000</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>２６冷やし中華</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>2532787000000</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>２６冷やし中華ミニ</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>2533587000000</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>２６冷やしきつねうどん</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>2551178000000</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>太麺ナポリタン２</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>2557960000000</t>
-        </is>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>関西風焼きそば３</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>2571104000000</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>２６きつねうどん</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>2571107000000</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>２６きつねうどん（小）</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>4522646118803</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Ｇ２６冷やし中華</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>4522646119046</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Ｇ２６冷やしきつねうどん</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>4522646138672</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Ｓ大盛ナポリタン</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>4522646138917</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Ｓ関西風オムそば３</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>4522646150544</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Ｓ太麺ナポリタン２</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
-        <is>
-          <t>4522646199468</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Ｇ関西風焼きそば３</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>4522646199475</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
           <t>Ｓ関西風焼きそば３</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
-        <is>
-          <t>4522646209709</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Ｇ２６きつねうどん</t>
         </is>
       </c>
     </row>

</xml_diff>